<commit_message>
statistics: income total, income by type. added high demand
</commit_message>
<xml_diff>
--- a/traffic_weather.xlsx
+++ b/traffic_weather.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ИРИТ\МАГА\1 курс\ProjectPracticeTaxi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10AC3DF6-D20A-4131-9B8F-FBBA6EA8C05B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9AEB44A-1DAC-47C2-8E69-44D5B3333459}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="300" yWindow="930" windowWidth="15330" windowHeight="14580" activeTab="3" xr2:uid="{82A27852-276A-433F-BB61-FC17B37C1351}"/>
+    <workbookView xWindow="14625" yWindow="450" windowWidth="14115" windowHeight="14580" activeTab="1" xr2:uid="{82A27852-276A-433F-BB61-FC17B37C1351}"/>
   </bookViews>
   <sheets>
     <sheet name="weekdaySnow" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="10">
   <si>
     <t>1.0</t>
   </si>
@@ -61,6 +61,12 @@
   </si>
   <si>
     <t>precipitationLevel</t>
+  </si>
+  <si>
+    <t>highDemand</t>
+  </si>
+  <si>
+    <t>true</t>
   </si>
 </sst>
 </file>
@@ -99,7 +105,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -137,11 +143,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -153,6 +185,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -487,14 +526,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE4B4DE6-7045-462E-86C7-97839848CDB9}">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="2" max="2" width="12.5" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="12.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="20.25" customHeight="1">
+    <row r="1" spans="1:4" ht="20.25" customHeight="1">
       <c r="A1" s="3" t="s">
         <v>5</v>
       </c>
@@ -504,8 +544,11 @@
       <c r="C1" s="4" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
+      <c r="D1" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" s="2">
         <v>0.29166666666666669</v>
       </c>
@@ -515,8 +558,9 @@
       <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:3">
+      <c r="D2" s="7"/>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" s="2">
         <v>0.33333333333333298</v>
       </c>
@@ -526,8 +570,9 @@
       <c r="C3" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:3">
+      <c r="D3" s="7"/>
+    </row>
+    <row r="4" spans="1:4">
       <c r="A4" s="2">
         <v>0.374999999999999</v>
       </c>
@@ -537,8 +582,9 @@
       <c r="C4" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:3">
+      <c r="D4" s="7"/>
+    </row>
+    <row r="5" spans="1:4">
       <c r="A5" s="2">
         <v>0.41666666666666602</v>
       </c>
@@ -548,8 +594,9 @@
       <c r="C5" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:3">
+      <c r="D5" s="7"/>
+    </row>
+    <row r="6" spans="1:4">
       <c r="A6" s="2">
         <v>0.45833333333333198</v>
       </c>
@@ -559,8 +606,9 @@
       <c r="C6" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="1:3">
+      <c r="D6" s="7"/>
+    </row>
+    <row r="7" spans="1:4">
       <c r="A7" s="2">
         <v>0.499999999999998</v>
       </c>
@@ -570,8 +618,9 @@
       <c r="C7" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="8" spans="1:3">
+      <c r="D7" s="7"/>
+    </row>
+    <row r="8" spans="1:4">
       <c r="A8" s="2">
         <v>0.54166666666666496</v>
       </c>
@@ -581,8 +630,9 @@
       <c r="C8" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="9" spans="1:3">
+      <c r="D8" s="7"/>
+    </row>
+    <row r="9" spans="1:4">
       <c r="A9" s="2">
         <v>0.58333333333333104</v>
       </c>
@@ -592,8 +642,11 @@
       <c r="C9" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="10" spans="1:3">
+      <c r="D9" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
       <c r="A10" s="2">
         <v>0.624999999999997</v>
       </c>
@@ -603,8 +656,11 @@
       <c r="C10" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="11" spans="1:3">
+      <c r="D10" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
       <c r="A11" s="2">
         <v>0.66666666666666397</v>
       </c>
@@ -614,8 +670,11 @@
       <c r="C11" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="12" spans="1:3">
+      <c r="D11" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
       <c r="A12" s="2">
         <v>0.70833333333333004</v>
       </c>
@@ -625,8 +684,11 @@
       <c r="C12" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="13" spans="1:3">
+      <c r="D12" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
       <c r="A13" s="2">
         <v>0.749999999999996</v>
       </c>
@@ -636,8 +698,11 @@
       <c r="C13" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="14" spans="1:3">
+      <c r="D13" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
       <c r="A14" s="2">
         <v>0.79166666666666297</v>
       </c>
@@ -647,8 +712,11 @@
       <c r="C14" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="15" spans="1:3">
+      <c r="D14" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
       <c r="A15" s="2">
         <v>0.83333333333332904</v>
       </c>
@@ -658,8 +726,11 @@
       <c r="C15" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:3">
+      <c r="D15" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
       <c r="A16" s="2">
         <v>0.874999999999995</v>
       </c>
@@ -668,6 +739,9 @@
       </c>
       <c r="C16" s="1" t="s">
         <v>3</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -677,14 +751,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2D54836-6042-4752-AF62-571232C81658}">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="2" max="2" width="13.25" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="11.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15">
+    <row r="1" spans="1:4" ht="15">
       <c r="A1" s="3" t="s">
         <v>5</v>
       </c>
@@ -694,8 +769,11 @@
       <c r="C1" s="4" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
+      <c r="D1" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" s="2">
         <v>0.29166666666666669</v>
       </c>
@@ -705,8 +783,9 @@
       <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:3">
+      <c r="D2" s="7"/>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" s="2">
         <v>0.33333333333333298</v>
       </c>
@@ -716,8 +795,9 @@
       <c r="C3" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="1:3">
+      <c r="D3" s="7"/>
+    </row>
+    <row r="4" spans="1:4">
       <c r="A4" s="2">
         <v>0.374999999999999</v>
       </c>
@@ -727,8 +807,9 @@
       <c r="C4" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:3">
+      <c r="D4" s="7"/>
+    </row>
+    <row r="5" spans="1:4">
       <c r="A5" s="2">
         <v>0.41666666666666602</v>
       </c>
@@ -738,8 +819,9 @@
       <c r="C5" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:3">
+      <c r="D5" s="7"/>
+    </row>
+    <row r="6" spans="1:4">
       <c r="A6" s="2">
         <v>0.45833333333333198</v>
       </c>
@@ -749,8 +831,9 @@
       <c r="C6" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="1:3">
+      <c r="D6" s="7"/>
+    </row>
+    <row r="7" spans="1:4">
       <c r="A7" s="2">
         <v>0.499999999999998</v>
       </c>
@@ -760,8 +843,9 @@
       <c r="C7" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="8" spans="1:3">
+      <c r="D7" s="7"/>
+    </row>
+    <row r="8" spans="1:4">
       <c r="A8" s="2">
         <v>0.54166666666666496</v>
       </c>
@@ -771,8 +855,9 @@
       <c r="C8" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="9" spans="1:3">
+      <c r="D8" s="7"/>
+    </row>
+    <row r="9" spans="1:4">
       <c r="A9" s="2">
         <v>0.58333333333333104</v>
       </c>
@@ -782,8 +867,9 @@
       <c r="C9" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="10" spans="1:3">
+      <c r="D9" s="7"/>
+    </row>
+    <row r="10" spans="1:4">
       <c r="A10" s="2">
         <v>0.624999999999997</v>
       </c>
@@ -793,8 +879,9 @@
       <c r="C10" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="11" spans="1:3">
+      <c r="D10" s="7"/>
+    </row>
+    <row r="11" spans="1:4">
       <c r="A11" s="2">
         <v>0.66666666666666397</v>
       </c>
@@ -804,8 +891,11 @@
       <c r="C11" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="12" spans="1:3">
+      <c r="D11" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
       <c r="A12" s="2">
         <v>0.70833333333333004</v>
       </c>
@@ -815,8 +905,11 @@
       <c r="C12" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="13" spans="1:3">
+      <c r="D12" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
       <c r="A13" s="2">
         <v>0.749999999999996</v>
       </c>
@@ -826,8 +919,11 @@
       <c r="C13" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="14" spans="1:3">
+      <c r="D13" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
       <c r="A14" s="2">
         <v>0.79166666666666297</v>
       </c>
@@ -837,8 +933,9 @@
       <c r="C14" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="15" spans="1:3">
+      <c r="D14" s="7"/>
+    </row>
+    <row r="15" spans="1:4">
       <c r="A15" s="2">
         <v>0.83333333333332904</v>
       </c>
@@ -848,8 +945,11 @@
       <c r="C15" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="16" spans="1:3">
+      <c r="D15" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
       <c r="A16" s="2">
         <v>0.874999999999995</v>
       </c>
@@ -858,6 +958,9 @@
       </c>
       <c r="C16" s="1" t="s">
         <v>3</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -867,187 +970,212 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5ED7BFF9-77A9-4DE5-B8A6-640507EC63DC}">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="2" max="2" width="12.375" customWidth="1"/>
     <col min="3" max="3" width="18.5" customWidth="1"/>
+    <col min="4" max="4" width="13.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15">
+    <row r="1" spans="1:4" ht="15">
       <c r="A1" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
+      <c r="D1" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" s="2">
         <v>0.29166666666666669</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
+      <c r="C2" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="7"/>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" s="2">
         <v>0.33333333333333298</v>
       </c>
       <c r="B3" s="1">
         <v>2</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="6" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:3">
+      <c r="D3" s="7"/>
+    </row>
+    <row r="4" spans="1:4">
       <c r="A4" s="2">
         <v>0.374999999999999</v>
       </c>
       <c r="B4" s="1">
         <v>2</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
+      <c r="C4" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="7"/>
+    </row>
+    <row r="5" spans="1:4">
       <c r="A5" s="2">
         <v>0.41666666666666602</v>
       </c>
       <c r="B5" s="1">
         <v>2</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
+      <c r="C5" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" s="7"/>
+    </row>
+    <row r="6" spans="1:4">
       <c r="A6" s="2">
         <v>0.45833333333333198</v>
       </c>
       <c r="B6" s="1">
         <v>2</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
+      <c r="C6" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="7"/>
+    </row>
+    <row r="7" spans="1:4">
       <c r="A7" s="2">
         <v>0.499999999999998</v>
       </c>
       <c r="B7" s="1">
         <v>3</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
+      <c r="C7" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7" s="7"/>
+    </row>
+    <row r="8" spans="1:4">
       <c r="A8" s="2">
         <v>0.54166666666666496</v>
       </c>
       <c r="B8" s="1">
         <v>4</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
+      <c r="C8" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" s="7"/>
+    </row>
+    <row r="9" spans="1:4">
       <c r="A9" s="2">
         <v>0.58333333333333104</v>
       </c>
       <c r="B9" s="1">
         <v>4</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
+      <c r="C9" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D9" s="7"/>
+    </row>
+    <row r="10" spans="1:4">
       <c r="A10" s="2">
         <v>0.624999999999997</v>
       </c>
       <c r="B10" s="1">
         <v>4</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
+      <c r="C10" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D10" s="7"/>
+    </row>
+    <row r="11" spans="1:4">
       <c r="A11" s="2">
         <v>0.66666666666666397</v>
       </c>
       <c r="B11" s="1">
         <v>3</v>
       </c>
-      <c r="C11" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3">
+      <c r="C11" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D11" s="7"/>
+    </row>
+    <row r="12" spans="1:4">
       <c r="A12" s="2">
         <v>0.70833333333333004</v>
       </c>
       <c r="B12" s="1">
         <v>3</v>
       </c>
-      <c r="C12" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3">
+      <c r="C12" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D12" s="7"/>
+    </row>
+    <row r="13" spans="1:4">
       <c r="A13" s="2">
         <v>0.749999999999996</v>
       </c>
       <c r="B13" s="1">
         <v>3</v>
       </c>
-      <c r="C13" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3">
+      <c r="C13" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D13" s="7"/>
+    </row>
+    <row r="14" spans="1:4">
       <c r="A14" s="2">
         <v>0.79166666666666297</v>
       </c>
       <c r="B14" s="1">
         <v>3</v>
       </c>
-      <c r="C14" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3">
+      <c r="C14" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
       <c r="A15" s="2">
         <v>0.83333333333332904</v>
       </c>
       <c r="B15" s="1">
         <v>3</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" s="6" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="16" spans="1:3">
+      <c r="D15" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
       <c r="A16" s="2">
         <v>0.874999999999995</v>
       </c>
       <c r="B16" s="1">
         <v>3</v>
       </c>
-      <c r="C16" s="1" t="s">
-        <v>3</v>
+      <c r="C16" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -1057,187 +1185,208 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F53F0B38-6217-49F9-88BA-6E3435233160}">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="2" max="2" width="13" customWidth="1"/>
     <col min="3" max="3" width="18.375" customWidth="1"/>
+    <col min="4" max="4" width="13.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15">
+    <row r="1" spans="1:4" ht="15">
       <c r="A1" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
+      <c r="D1" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" s="2">
         <v>0.29166666666666669</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
+      <c r="C2" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="7"/>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" s="2">
         <v>0.33333333333333298</v>
       </c>
       <c r="B3" s="1">
         <v>2</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="6" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:3">
+      <c r="D3" s="7"/>
+    </row>
+    <row r="4" spans="1:4">
       <c r="A4" s="2">
         <v>0.374999999999999</v>
       </c>
       <c r="B4" s="1">
         <v>2</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
+      <c r="C4" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="7"/>
+    </row>
+    <row r="5" spans="1:4">
       <c r="A5" s="2">
         <v>0.41666666666666602</v>
       </c>
       <c r="B5" s="1">
         <v>3</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
+      <c r="C5" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" s="7"/>
+    </row>
+    <row r="6" spans="1:4">
       <c r="A6" s="2">
         <v>0.45833333333333198</v>
       </c>
       <c r="B6" s="1">
         <v>4</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
+      <c r="C6" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="7"/>
+    </row>
+    <row r="7" spans="1:4">
       <c r="A7" s="2">
         <v>0.499999999999998</v>
       </c>
       <c r="B7" s="1">
         <v>5</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
+      <c r="C7" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7" s="7"/>
+    </row>
+    <row r="8" spans="1:4">
       <c r="A8" s="2">
         <v>0.54166666666666496</v>
       </c>
       <c r="B8" s="1">
         <v>5</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
+      <c r="C8" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" s="7"/>
+    </row>
+    <row r="9" spans="1:4">
       <c r="A9" s="2">
         <v>0.58333333333333104</v>
       </c>
       <c r="B9" s="1">
         <v>5</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
+      <c r="C9" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D9" s="7"/>
+    </row>
+    <row r="10" spans="1:4">
       <c r="A10" s="2">
         <v>0.624999999999997</v>
       </c>
       <c r="B10" s="1">
         <v>6</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
+      <c r="C10" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D10" s="7"/>
+    </row>
+    <row r="11" spans="1:4">
       <c r="A11" s="2">
         <v>0.66666666666666397</v>
       </c>
       <c r="B11" s="1">
         <v>5</v>
       </c>
-      <c r="C11" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3">
+      <c r="C11" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D11" s="7"/>
+    </row>
+    <row r="12" spans="1:4">
       <c r="A12" s="2">
         <v>0.70833333333333004</v>
       </c>
       <c r="B12" s="1">
         <v>4</v>
       </c>
-      <c r="C12" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3">
+      <c r="C12" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D12" s="7"/>
+    </row>
+    <row r="13" spans="1:4">
       <c r="A13" s="2">
         <v>0.749999999999996</v>
       </c>
       <c r="B13" s="1">
         <v>4</v>
       </c>
-      <c r="C13" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3">
+      <c r="C13" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D13" s="7"/>
+    </row>
+    <row r="14" spans="1:4">
       <c r="A14" s="2">
         <v>0.79166666666666297</v>
       </c>
       <c r="B14" s="1">
         <v>3</v>
       </c>
-      <c r="C14" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3">
+      <c r="C14" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D14" s="7"/>
+    </row>
+    <row r="15" spans="1:4">
       <c r="A15" s="2">
         <v>0.83333333333332904</v>
       </c>
       <c r="B15" s="1">
         <v>3</v>
       </c>
-      <c r="C15" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3">
+      <c r="C15" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D15" s="7"/>
+    </row>
+    <row r="16" spans="1:4">
       <c r="A16" s="2">
         <v>0.874999999999995</v>
       </c>
       <c r="B16" s="1">
         <v>3</v>
       </c>
-      <c r="C16" s="1" t="s">
-        <v>3</v>
+      <c r="C16" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>